<commit_message>
Added README and requirement
</commit_message>
<xml_diff>
--- a/grid_analysis_log.xlsx
+++ b/grid_analysis_log.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC140"/>
+  <dimension ref="A1:AC141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12852,6 +12852,105 @@
         <v>62.4</v>
       </c>
     </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2026-06-14 23</t>
+        </is>
+      </c>
+      <c r="B141" t="n">
+        <v>49.8</v>
+      </c>
+      <c r="C141" t="n">
+        <v>77027.64646434024</v>
+      </c>
+      <c r="D141" t="n">
+        <v>80879.03</v>
+      </c>
+      <c r="E141" t="n">
+        <v>225</v>
+      </c>
+      <c r="F141" t="n">
+        <v>11</v>
+      </c>
+      <c r="G141" t="n">
+        <v>0.8661580944054629</v>
+      </c>
+      <c r="H141" t="n">
+        <v>1526.002460166704</v>
+      </c>
+      <c r="I141" t="n">
+        <v>3053.408861587021</v>
+      </c>
+      <c r="J141" t="n">
+        <v>60.5</v>
+      </c>
+      <c r="K141" t="n">
+        <v>97.55555555555556</v>
+      </c>
+      <c r="L141" t="n">
+        <v>25</v>
+      </c>
+      <c r="M141" t="n">
+        <v>3851.383535659756</v>
+      </c>
+      <c r="N141" t="n">
+        <v>95.23809381039837</v>
+      </c>
+      <c r="O141" t="n">
+        <v>88.30790472027314</v>
+      </c>
+      <c r="P141" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="Q141" t="n">
+        <v>50</v>
+      </c>
+      <c r="R141" t="n">
+        <v>50</v>
+      </c>
+      <c r="S141" t="n">
+        <v>85.30790472027314</v>
+      </c>
+      <c r="T141" t="n">
+        <v>80.30790472027314</v>
+      </c>
+      <c r="U141" t="n">
+        <v>55.00000000000001</v>
+      </c>
+      <c r="V141" t="n">
+        <v>75</v>
+      </c>
+      <c r="W141" t="inlineStr">
+        <is>
+          <t>High Grid Stress</t>
+        </is>
+      </c>
+      <c r="X141" t="inlineStr">
+        <is>
+          <t>Perform load balancing</t>
+        </is>
+      </c>
+      <c r="Y141" t="n">
+        <v>640</v>
+      </c>
+      <c r="Z141" t="n">
+        <v>33</v>
+      </c>
+      <c r="AA141" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB141" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="AC141" t="n">
+        <v>64.7</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>